<commit_message>
changes for ABP-Demo-Successfull Payment
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="109">
   <si>
     <t>BillType</t>
   </si>
@@ -427,6 +427,57 @@
   </si>
   <si>
     <t>Mon Dec 15 16:30:22 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:07:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:08:14 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:08:35 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:10:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:11:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:11:42 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:12:24 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:13:05 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:13:52 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:16:46 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:17:29 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:18:11 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:19:06 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:20:38 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:21:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:21:49 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Dec 26 20:22:27 IST 2025</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1082,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1106,7 +1157,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1199,7 +1250,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1274,7 +1325,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1345,7 +1396,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1438,7 +1489,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1534,7 +1585,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1614,7 +1665,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1669,7 +1720,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1736,7 +1787,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1873,10 +1924,10 @@
     </row>
     <row ht="232" r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2236,7 +2287,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2290,10 +2341,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2335,7 +2386,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>103</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2387,7 +2438,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2408,7 +2459,7 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -2425,7 +2476,7 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
chnages with ABP QA & Demo
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="110">
   <si>
     <t>BillType</t>
   </si>
@@ -478,6 +478,9 @@
   </si>
   <si>
     <t>Fri Dec 26 20:22:27 IST 2025</t>
+  </si>
+  <si>
+    <t>Fri Jan 09 17:02:29 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -2341,10 +2344,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">

</xml_diff>

<commit_message>
Bill File Lookup TCs on Demo server
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="134">
   <si>
     <t>BillType</t>
   </si>
@@ -481,6 +481,78 @@
   </si>
   <si>
     <t>Fri Jan 09 17:02:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:21:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:22:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:22:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:24:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:25:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:25:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:26:38 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:27:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:28:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:31:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:31:40 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:32:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:33:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:34:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:35:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:35:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 02:36:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 21:25:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 21:27:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 21:29:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 21:30:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 21:32:54 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 22:35:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Mar 10 22:40:41 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1085,7 +1157,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1160,7 +1232,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1253,7 +1325,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1328,7 +1400,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1399,7 +1471,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1492,7 +1564,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1588,7 +1660,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1668,7 +1740,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1723,7 +1795,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1790,7 +1862,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1930,7 +2002,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2290,7 +2362,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2347,7 +2419,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2389,7 +2461,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2441,7 +2513,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2462,7 +2534,7 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -2479,7 +2551,7 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
Manual Entry page chnages for Demo & Prod servers
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="152">
   <si>
     <t>BillType</t>
   </si>
@@ -553,6 +553,60 @@
   </si>
   <si>
     <t>Tue Mar 10 22:40:41 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 10:56:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 10:57:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 10:57:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 10:59:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:00:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:00:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:01:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:01:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:02:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:05:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:05:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:06:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:07:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:08:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:09:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:09:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:10:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 17:28:26 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1154,10 +1208,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1232,7 +1286,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1325,7 +1379,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1400,7 +1454,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1471,7 +1525,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1564,7 +1618,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1660,7 +1714,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1740,7 +1794,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1795,7 +1849,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1862,7 +1916,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2002,7 +2056,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2362,7 +2416,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2419,7 +2473,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2461,7 +2515,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2513,7 +2567,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2534,7 +2588,7 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -2551,7 +2605,7 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
ABP Regression on QA server
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t470258\Documents\VPS-Katalon\KatalonData\ABPTestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{57A52135-CCF2-4101-8516-0F507AB366ED}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr documentId="13_ncr:1_{E1567607-66D6-4773-9C66-B0D9B77FBB24}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView activeTab="19" firstSheet="18" windowHeight="11500" windowWidth="19420" xWindow="-110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-110"/>
+    <workbookView activeTab="9" firstSheet="7" windowHeight="11500" windowWidth="19420" xWindow="-110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-110"/>
   </bookViews>
   <sheets>
     <sheet name="UIVerification-RegisterPayPage" r:id="rId1" sheetId="1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="88">
   <si>
     <t>BillType</t>
   </si>
@@ -234,9 +234,6 @@
     <t>Password must be at least 8 characters long and no more than 32 characters long.,Password must contain at least one alpha character and one numeric character.,The password must also contain at least one special character.</t>
   </si>
   <si>
-    <t>Username must be at least 6 characters long.</t>
-  </si>
-  <si>
     <t>UserName</t>
   </si>
   <si>
@@ -360,253 +357,64 @@
 Individual Amount:,Repeat this amount until the Balance Due is achieved: $,1 Annual payment of $10.00 on </t>
   </si>
   <si>
-    <t>Thu Oct 30 10:51:41 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:52:02 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:52:21 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:53:59 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:54:45 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:55:02 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:55:41 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:56:31 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 10:59:53 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 11:00:34 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 11:01:45 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 11:03:22 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 11:03:52 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 11:04:22 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 11:04:53 IST 2025</t>
-  </si>
-  <si>
-    <t>Thu Oct 30 21:46:17 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Oct 31 21:00:36 IST 2025</t>
+    <t>Tue Jun 02 10:57:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 10:57:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 10:59:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:00:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:00:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:01:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:01:52 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:02:29 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:05:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:05:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:06:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:07:14 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:08:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:09:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Jun 02 11:09:50 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jun 05 18:22:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jun 05 18:45:13 IST 2026</t>
+  </si>
+  <si>
+    <t>Please choose another user name</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Fri Dec 12 16:53:57 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 12 17:45:47 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 12 18:44:21 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 12 18:47:10 IST 2025</t>
-  </si>
-  <si>
-    <t>Mon Dec 15 16:30:22 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:07:52 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:08:14 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:08:35 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:10:29 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:11:17 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:11:42 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:12:24 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:13:05 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:13:52 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:16:46 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:17:29 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:18:11 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:19:06 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:20:38 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:21:17 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:21:49 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Dec 26 20:22:27 IST 2025</t>
-  </si>
-  <si>
-    <t>Fri Jan 09 17:02:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:21:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:22:38 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:22:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:24:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:25:34 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:25:56 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:26:38 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:27:20 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:28:03 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:31:01 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:31:40 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:32:19 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:33:13 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:34:43 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:35:17 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:35:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 02:36:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 21:25:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 21:27:17 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 21:29:02 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 21:30:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 21:32:54 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 22:35:05 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Mar 10 22:40:41 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 10:56:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 10:57:27 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 10:57:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 10:59:23 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:00:05 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:00:24 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:01:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:01:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:02:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:05:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:05:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:06:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:07:14 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:08:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:09:20 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:09:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:10:19 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 17:28:26 IST 2026</t>
+    <t>Fri Jun 05 18:51:13 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1203,15 +1011,15 @@
         <v>10</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>150</v>
+        <v>87</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1221,7 +1029,7 @@
         <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
@@ -1260,7 +1068,7 @@
         <v>10</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H1" s="13" t="s">
         <v>16</v>
@@ -1286,7 +1094,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>68</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1296,19 +1104,19 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" t="s">
         <v>52</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>53</v>
-      </c>
-      <c r="J2" t="s">
-        <v>54</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>23</v>
@@ -1353,7 +1161,7 @@
         <v>10</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H1" s="13" t="s">
         <v>16</v>
@@ -1379,7 +1187,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>83</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1389,19 +1197,19 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" t="s">
         <v>52</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>53</v>
-      </c>
-      <c r="J2" t="s">
-        <v>54</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>23</v>
@@ -1446,7 +1254,7 @@
         <v>10</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row ht="116" r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1454,7 +1262,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>71</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1464,7 +1272,7 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
@@ -1502,7 +1310,7 @@
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>5</v>
@@ -1511,13 +1319,13 @@
         <v>25</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row ht="362.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -1525,7 +1333,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1535,11 +1343,11 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>11/04/2025</v>
+        <v>06/06/2026</v>
       </c>
       <c r="H2" s="18">
         <v>10</v>
@@ -1556,11 +1364,11 @@
 Number of Payments:,Divide the Balance Due into ,
 Individual Amount:,Repeat this amount until the Balance Due is achieved: $, 
 Step 4: Review Payment Plan,
-1 Daily payment of $10.00 on 11/04/2025,A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 11/04/2025</v>
+1 Daily payment of $10.00 on 06/06/2026,A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 06/06/2026</v>
       </c>
       <c r="K2" s="14" t="str">
         <f ca="1">"A Convenience Fee will be added to each transaction issued for 1 Daily payment of "&amp;  TEXT(I2,"0.00")&amp;" starting on "&amp;G2</f>
-        <v>A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 11/04/2025</v>
+        <v>A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 06/06/2026</v>
       </c>
     </row>
   </sheetData>
@@ -1595,7 +1403,7 @@
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>5</v>
@@ -1604,13 +1412,13 @@
         <v>25</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row ht="304.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -1618,7 +1426,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>77</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1628,11 +1436,11 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>11/04/2025</v>
+        <v>06/06/2026</v>
       </c>
       <c r="H2" s="18">
         <v>10</v>
@@ -1646,7 +1454,7 @@
 Deferred,
 Select the date you wish to submit your payment,
 Step 4: Review Payment Plan,
-1 Deferred payment of $10.00 on 11/04/2025,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 11/04/2025 ,Individual Convenience Fee Amount:,	
+1 Deferred payment of $10.00 on 06/06/2026,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
@@ -1654,7 +1462,7 @@
         <f ca="1">"A Convenience Fee will be added to each transaction issued for 1 Deferred payment of "&amp;  TEXT(I2,"0.00")&amp;" starting on "&amp;G2&amp;" ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:"</f>
-        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 11/04/2025 ,Individual Convenience Fee Amount:,	
+        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
@@ -1691,7 +1499,7 @@
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>5</v>
@@ -1700,13 +1508,13 @@
         <v>25</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J1" s="13" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row ht="304.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -1714,7 +1522,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1724,11 +1532,11 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>11/04/2025</v>
+        <v>06/06/2026</v>
       </c>
       <c r="H2" s="18">
         <v>10</v>
@@ -1743,7 +1551,7 @@
 Daily,
 Select the date you wish to submit your first payment and it will recur every day after,
 Step 4: Review Payment Plan,
-Daily payments of $10.00 starting on 11/04/2025,A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 11/04/2025 ,Individual Convenience Fee Amount:,	
+Daily payments of $10.00 starting on 06/06/2026,A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
@@ -1751,7 +1559,7 @@
         <f ca="1">"A Convenience Fee will be added to each transaction issued for Daily payment of "&amp;  TEXT(I2,"0.00")&amp;" starting on "&amp;G2&amp;" ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:"</f>
-        <v>A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 11/04/2025 ,Individual Convenience Fee Amount:,	
+        <v>A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
@@ -1794,7 +1602,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1804,7 +1612,7 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1838,7 +1646,7 @@
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>10</v>
@@ -1849,7 +1657,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>141</v>
+        <v>74</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1859,7 +1667,7 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G2" s="14" t="str">
         <f ca="1">F2&amp;TEXT(TODAY()+1,"mm/dd/yyyy")</f>
@@ -1871,7 +1679,7 @@
 Number of Payments:,Divide the Balance Due into, 
 Individual Amount:,	Repeat this amount until the Balance Due is achieved: $ ,
 Step 4: Review Payment Plan
-1 Quarterly payment of $10.00 on 11/04/2025</v>
+1 Quarterly payment of $10.00 on 06/06/2026</v>
       </c>
     </row>
   </sheetData>
@@ -1905,7 +1713,7 @@
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>10</v>
@@ -1916,7 +1724,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>72</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1926,7 +1734,7 @@
         <v>43</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G2" s="16" t="str">
         <f ca="1">F2&amp;TEXT(TODAY()+1,"mm/dd/yyyy")</f>
@@ -1935,7 +1743,7 @@
 Select the date you wish to submit your first payment and it will recur every year on that day,
 Divide your payment plan by...,
 Number of Payments:,Divide the Balance Due into,
-Individual Amount:,Repeat this amount until the Balance Due is achieved: $,1 Annual payment of $10.00 on 11/04/2025</v>
+Individual Amount:,Repeat this amount until the Balance Due is achieved: $,1 Annual payment of $10.00 on 06/06/2026</v>
       </c>
     </row>
   </sheetData>
@@ -2033,7 +1841,7 @@
         <v>7</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>5</v>
@@ -2042,13 +1850,13 @@
         <v>25</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I1" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row ht="232" r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -2056,18 +1864,18 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
+        <v>75</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>11/04/2025</v>
+        <v>06/06/2026</v>
       </c>
       <c r="G2" s="18">
         <v>10</v>
@@ -2083,11 +1891,11 @@
  Individual Amount:,	Repeat this amount until the Balance Due is achieved: $, 
 10.00,
 Step 4: Review Payment Plan,
-1 Deferred payment of $10.00 on 11/04/2025,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 11/04/2025</v>
+1 Deferred payment of $10.00 on 06/06/2026,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026</v>
       </c>
       <c r="J2" s="14" t="str">
         <f ca="1">"A Convenience Fee will be added to each transaction issued for 1 Deferred payment of "&amp;  TEXT(H2,"0.00")&amp;" starting on "&amp;F2</f>
-        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 11/04/2025</v>
+        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026</v>
       </c>
     </row>
   </sheetData>
@@ -2416,7 +2224,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>69</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2473,7 +2281,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>79</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2515,7 +2323,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>145</v>
+        <v>78</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2567,7 +2375,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>147</v>
+        <v>80</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2588,7 +2396,7 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>148</v>
+        <v>81</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -2605,7 +2413,7 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>149</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
EmailTextToPay execution on Upgrade
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="116">
   <si>
     <t>BillType</t>
   </si>
@@ -496,6 +496,9 @@
   </si>
   <si>
     <t>Fri Jun 19 11:16:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 03 04:39:58 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -932,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="17.0" collapsed="true"/>
@@ -1035,7 +1038,7 @@
       <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -1050,7 +1053,7 @@
       <c r="H3" s="1">
         <v>300002</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" t="s" s="0">
         <v>12</v>
       </c>
     </row>
@@ -1064,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A409B366-E307-4873-AD1A-14C5ECF78921}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="19.08984375" collapsed="true"/>
@@ -1096,10 +1099,10 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>114</v>
       </c>
       <c r="C2" s="12"/>
@@ -1109,10 +1112,10 @@
       <c r="E2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
     </row>
@@ -1123,7 +1126,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33DFE7B9-88F3-4E87-BB56-955EB38799F0}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="53.36328125" collapsed="true"/>
@@ -1171,11 +1174,11 @@
       </c>
     </row>
     <row ht="261" r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
-        <v>89</v>
+      <c r="B2" t="s" s="0">
+        <v>115</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1187,25 +1190,25 @@
       <c r="F2" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>53</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="0">
         <v>20770</v>
       </c>
     </row>
@@ -1216,7 +1219,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51EBD9BD-D9A5-41D7-B0D1-A7DD8841A698}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="39.7265625" collapsed="true"/>
@@ -1264,10 +1267,10 @@
       </c>
     </row>
     <row ht="159.5" r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>88</v>
       </c>
       <c r="C2" s="12"/>
@@ -1280,25 +1283,25 @@
       <c r="F2" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>53</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="0">
         <v>20770</v>
       </c>
     </row>
@@ -1309,7 +1312,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DDB5A32-AE5F-4469-909E-B5CBB0B316F1}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="44.26953125" collapsed="true"/>
@@ -1339,10 +1342,10 @@
       </c>
     </row>
     <row ht="116" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>92</v>
       </c>
       <c r="C2" s="12"/>
@@ -1355,7 +1358,7 @@
       <c r="F2" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
     </row>
@@ -1366,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDED305E-1D1F-4473-A9FE-10CCE4EF2A93}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="34.36328125" collapsed="true"/>
@@ -1410,10 +1413,10 @@
       </c>
     </row>
     <row ht="362.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>106</v>
       </c>
       <c r="C2" s="12"/>
@@ -1459,7 +1462,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4382B992-23F5-4C47-8E0D-617770DAB873}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="27.6328125" collapsed="true"/>
@@ -1503,10 +1506,10 @@
       </c>
     </row>
     <row ht="304.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>110</v>
       </c>
       <c r="C2" s="12"/>
@@ -1555,7 +1558,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EA3BF1-14B8-47AF-A2C8-3C7ED7468772}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="29.90625" collapsed="true"/>
@@ -1599,10 +1602,10 @@
       </c>
     </row>
     <row ht="304.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>109</v>
       </c>
       <c r="C2" s="12"/>
@@ -1652,7 +1655,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E59FD46A-A4BF-4EFF-8C85-302E7420C761}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="40.54296875" collapsed="true"/>
@@ -1679,10 +1682,10 @@
       </c>
     </row>
     <row ht="101.5" r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>91</v>
       </c>
       <c r="C2" s="12"/>
@@ -1703,7 +1706,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D81D62B-D7FF-4418-A543-2CCEB8B27904}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="39.453125" collapsed="true"/>
@@ -1734,10 +1737,10 @@
       </c>
     </row>
     <row ht="246.5" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>107</v>
       </c>
       <c r="C2" s="12"/>
@@ -1770,7 +1773,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6951466-0A68-4F4C-8CFE-91C88774BAFD}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" customWidth="true" width="53.6328125" collapsed="true"/>
@@ -1801,10 +1804,10 @@
       </c>
     </row>
     <row ht="159.5" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>105</v>
       </c>
       <c r="C2" s="12"/>
@@ -1834,7 +1837,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F59C5AD-9583-4572-BF59-08E264185AA4}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" bestFit="true" customWidth="true" width="9.81640625" collapsed="true"/>
@@ -1877,16 +1880,16 @@
       <c r="C2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="0">
         <v>1</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="0">
         <v>1</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="0">
         <v>3</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="0">
         <v>6</v>
       </c>
     </row>
@@ -1897,7 +1900,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{106EA5F4-3A74-4B88-9694-190DD754DB42}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" customWidth="true" width="35.54296875" collapsed="true"/>
@@ -1941,10 +1944,10 @@
       </c>
     </row>
     <row ht="232" r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>108</v>
       </c>
       <c r="C2" s="12"/>
@@ -1986,7 +1989,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22FCBBA-7D6F-4A96-ABDF-B9688B9AD57A}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="25.7265625" collapsed="true"/>
@@ -2030,10 +2033,10 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>36</v>
       </c>
       <c r="C2" s="4"/>
@@ -2061,10 +2064,10 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>37</v>
       </c>
       <c r="C3" s="4"/>
@@ -2088,10 +2091,10 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>38</v>
       </c>
       <c r="C4" s="4"/>
@@ -2121,7 +2124,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2E036A-EB5C-429E-B5B6-2CEB663A49DE}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="25.81640625" collapsed="true"/>
@@ -2160,10 +2163,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>40</v>
       </c>
       <c r="C2" s="4"/>
@@ -2196,7 +2199,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8A1DA2-5F25-403C-A696-AD0A990EA2A5}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row ht="29" r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -2232,10 +2235,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C2" s="4"/>
@@ -2268,7 +2271,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3003305-5779-4E10-BB96-1E05DA55CF7C}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -2301,10 +2304,10 @@
       </c>
     </row>
     <row ht="409.5" r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>90</v>
       </c>
       <c r="C2" s="12"/>
@@ -2334,7 +2337,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8EB073-2CB6-4360-AD8F-5A1F832738F2}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" bestFit="true" customWidth="true" width="19.08984375" collapsed="true"/>
@@ -2358,10 +2361,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>100</v>
       </c>
       <c r="C2" s="12"/>
@@ -2379,7 +2382,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F658B4C-7DBB-4EDF-981E-97E4B7C1F375}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -2400,10 +2403,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>112</v>
       </c>
       <c r="C2" s="12"/>
@@ -2421,7 +2424,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C921207-0810-405F-8F16-4133FFE6EA23}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="6" bestFit="true" customWidth="true" width="19.08984375" collapsed="true"/>
@@ -2452,10 +2455,10 @@
       </c>
     </row>
     <row customHeight="1" ht="52" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>101</v>
       </c>
       <c r="C2" s="12"/>
@@ -2465,7 +2468,7 @@
       <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="G2" s="14" t="s">
@@ -2473,16 +2476,16 @@
       </c>
     </row>
     <row ht="29" r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>102</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>45</v>
       </c>
       <c r="G3" s="14" t="s">
@@ -2490,19 +2493,19 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>103</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>48</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="0">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
User List for ABP Demo
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="134">
   <si>
     <t>BillType</t>
   </si>
@@ -499,6 +499,60 @@
   </si>
   <si>
     <t>Fri Jul 03 04:39:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Aug 06 11:25:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Aug 06 11:25:39 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Aug 06 11:25:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Aug 06 11:27:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Aug 06 11:28:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 01:03:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 01:04:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 01:04:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 01:05:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 01:06:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:27:58 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:28:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:29:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:32:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:32:48 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:34:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:34:47 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 08 19:35:16 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1175,10 +1229,10 @@
     </row>
     <row ht="261" r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1271,7 +1325,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1346,7 +1400,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1417,7 +1471,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1510,7 +1564,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1606,7 +1660,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1686,7 +1740,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1741,7 +1795,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1948,7 +2002,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2308,7 +2362,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2459,7 +2513,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2480,7 +2534,7 @@
         <v>34</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>8</v>
@@ -2497,7 +2551,7 @@
         <v>34</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>8</v>

</xml_diff>

<commit_message>
user list page for ABP
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/ABPTestData.xlsx
+++ b/KatalonData/ABPTestData/ABPTestData.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t470258\Documents\VPS-Katalon\KatalonData\ABPTestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{E1567607-66D6-4773-9C66-B0D9B77FBB24}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3275BD-5542-4BE7-B2A1-064DB90EE424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="9" firstSheet="7" windowHeight="11500" windowWidth="19420" xWindow="-110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" yWindow="-110"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="UIVerification-RegisterPayPage" r:id="rId1" sheetId="1"/>
-    <sheet name="Sheet1" r:id="rId2" sheetId="2"/>
-    <sheet name="SuccessfulPaymentCC" r:id="rId3" sheetId="3"/>
-    <sheet name="VerifySuccessfulPaymentPSNoCF" r:id="rId4" sheetId="4"/>
-    <sheet name="VerifySuccessfulPaymentCorpNoCF" r:id="rId5" sheetId="5"/>
-    <sheet name="UIVerificationPendingBillsPage" r:id="rId6" sheetId="6"/>
-    <sheet name="CreateDeleteProfileOwner" r:id="rId7" sheetId="7"/>
-    <sheet name="CreateDeletePayer" r:id="rId8" sheetId="8"/>
-    <sheet name="VerifyPasswordPolicy" r:id="rId9" sheetId="9"/>
-    <sheet name="VerifyUsernameLength" r:id="rId10" sheetId="10"/>
-    <sheet name="UiVerificationForAddUser" r:id="rId11" sheetId="11"/>
-    <sheet name="UiVerificationForAccountProfile" r:id="rId12" sheetId="20"/>
-    <sheet name="UiVerificationSPBillsLabel" r:id="rId13" sheetId="12"/>
-    <sheet name="UiVerificationSPIPDaily" r:id="rId14" sheetId="13"/>
-    <sheet name="UiVerificationSPRecDeferred" r:id="rId15" sheetId="17"/>
-    <sheet name="UiVerificationSPRecDaily" r:id="rId16" sheetId="19"/>
-    <sheet name="UiVerificationSPAP" r:id="rId17" sheetId="18"/>
-    <sheet name="UiVerificationSPInstallmentQuar" r:id="rId18" sheetId="14"/>
-    <sheet name="UiVerificationSPInstallmentAnua" r:id="rId19" sheetId="15"/>
-    <sheet name="UiVerificationSPIPDeferred" r:id="rId20" sheetId="16"/>
+    <sheet name="UIVerification-RegisterPayPage" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="SuccessfulPaymentCC" sheetId="3" r:id="rId3"/>
+    <sheet name="VerifySuccessfulPaymentPSNoCF" sheetId="4" r:id="rId4"/>
+    <sheet name="VerifySuccessfulPaymentCorpNoCF" sheetId="5" r:id="rId5"/>
+    <sheet name="UIVerificationPendingBillsPage" sheetId="6" r:id="rId6"/>
+    <sheet name="CreateDeleteProfileOwner" sheetId="7" r:id="rId7"/>
+    <sheet name="CreateDeletePayer" sheetId="8" r:id="rId8"/>
+    <sheet name="VerifyPasswordPolicy" sheetId="9" r:id="rId9"/>
+    <sheet name="VerifyUsernameLength" sheetId="10" r:id="rId10"/>
+    <sheet name="UiVerificationForAddUser" sheetId="11" r:id="rId11"/>
+    <sheet name="UiVerificationForAccountProfile" sheetId="20" r:id="rId12"/>
+    <sheet name="UiVerificationSPBillsLabel" sheetId="12" r:id="rId13"/>
+    <sheet name="UiVerificationSPIPDaily" sheetId="13" r:id="rId14"/>
+    <sheet name="UiVerificationSPRecDeferred" sheetId="17" r:id="rId15"/>
+    <sheet name="UiVerificationSPRecDaily" sheetId="19" r:id="rId16"/>
+    <sheet name="UiVerificationSPAP" sheetId="18" r:id="rId17"/>
+    <sheet name="UiVerificationSPInstallmentQuar" sheetId="14" r:id="rId18"/>
+    <sheet name="UiVerificationSPInstallmentAnua" sheetId="15" r:id="rId19"/>
+    <sheet name="UiVerificationSPIPDeferred" sheetId="16" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="86">
   <si>
     <t>BillType</t>
   </si>
@@ -357,202 +357,58 @@
 Individual Amount:,Repeat this amount until the Balance Due is achieved: $,1 Annual payment of $10.00 on </t>
   </si>
   <si>
-    <t>Tue Jun 02 10:57:27 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 10:57:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 10:59:23 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:00:05 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:00:24 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:01:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:01:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:02:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:05:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:05:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:06:21 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:07:14 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:08:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:09:20 IST 2026</t>
-  </si>
-  <si>
-    <t>Tue Jun 02 11:09:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 05 18:22:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 05 18:45:13 IST 2026</t>
-  </si>
-  <si>
     <t>Please choose another user name</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Fri Jun 05 18:51:13 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:32:41 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:33:06 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:33:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:35:35 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:36:19 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:36:45 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:37:31 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:38:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:39:03 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:42:10 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:43:02 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:43:45 IST 2026</t>
-  </si>
-  <si>
     <t>Fri Jun 19 01:44:23 IST 2026</t>
   </si>
   <si>
-    <t>Fri Jun 19 01:51:26 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:52:10 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:52:46 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 01:53:22 IST 2026</t>
-  </si>
-  <si>
     <t>Fri Jun 19 10:56:21 IST 2026</t>
   </si>
   <si>
-    <t>Fri Jun 19 10:59:00 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 11:00:33 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 11:02:09 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 11:04:22 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 11:05:50 IST 2026</t>
-  </si>
-  <si>
-    <t>Fri Jun 19 11:07:18 IST 2026</t>
-  </si>
-  <si>
     <t>Fri Jun 19 11:09:58 IST 2026</t>
   </si>
   <si>
-    <t>Fri Jun 19 11:15:01 IST 2026</t>
-  </si>
-  <si>
     <t>Fri Jun 19 11:16:21 IST 2026</t>
   </si>
   <si>
-    <t>Fri Jul 03 04:39:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Aug 06 11:25:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Aug 06 11:25:39 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Aug 06 11:25:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Aug 06 11:27:25 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Aug 06 11:28:04 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 01:03:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 01:04:03 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 01:04:18 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 01:05:26 IST 2026</t>
-  </si>
-  <si>
     <t>Sat Aug 08 01:06:02 IST 2026</t>
   </si>
   <si>
-    <t>Sat Aug 08 19:27:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:28:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:29:37 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:32:11 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:32:48 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:34:17 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:34:47 IST 2026</t>
-  </si>
-  <si>
-    <t>Sat Aug 08 19:35:16 IST 2026</t>
+    <t>Fri Aug 14 23:00:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Aug 14 23:00:35 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Aug 14 23:00:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Aug 14 23:01:59 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 15 00:45:27 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 15 00:46:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 15 00:47:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 15 00:48:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Sat Aug 15 00:48:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Aug 19 17:42:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Aug 19 17:44:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Aug 19 17:46:30 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -653,68 +509,71 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
+  <cellXfs count="20">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="2" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
-    <xf applyAlignment="1" applyBorder="1" applyFont="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyFill="1" applyFont="1" borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="3" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="4" fillId="0" fontId="0" numFmtId="49" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="2" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="164" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -731,10 +590,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -769,7 +628,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin panose="020F0302020204030204" typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -804,7 +663,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin panose="020F0502020204030204" typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -898,21 +757,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="6350">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -929,7 +788,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -981,23 +840,23 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" name="Office Theme" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0" collapsed="true"/>
-    <col min="6" max="8" bestFit="true" customWidth="true" width="11.81640625" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" width="16.6328125" collapsed="true"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="9.26953125" collapsed="true"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="13.7265625" collapsed="true"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="11.90625" collapsed="true"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="8" width="11.81640625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="16.6328125" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="9.26953125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="12" max="12" width="13.7265625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="13" max="13" width="11.90625" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
@@ -1050,7 +909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row ht="409.5" r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="409.5" x14ac:dyDescent="0.35">
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4" t="s">
@@ -1092,7 +951,7 @@
       <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -1107,12 +966,12 @@
       <c r="H3" s="1">
         <v>300002</v>
       </c>
-      <c r="I3" t="s" s="0">
+      <c r="I3" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
@@ -1120,13 +979,13 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A409B366-E307-4873-AD1A-14C5ECF78921}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A409B366-E307-4873-AD1A-14C5ECF78921}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="19.08984375" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="38.7265625" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" width="10.7265625" collapsed="true"/>
+    <col min="5" max="5" width="19.08984375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="38.7265625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1153,11 +1012,11 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>114</v>
+      <c r="B2" t="s">
+        <v>72</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1166,27 +1025,27 @@
       <c r="E2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F2" t="s" s="0">
-        <v>85</v>
-      </c>
-      <c r="G2" t="s" s="0">
+      <c r="F2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33DFE7B9-88F3-4E87-BB56-955EB38799F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33DFE7B9-88F3-4E87-BB56-955EB38799F0}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="53.36328125" collapsed="true"/>
+    <col min="6" max="6" width="53.36328125" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1227,12 +1086,12 @@
         <v>18</v>
       </c>
     </row>
-    <row ht="261" r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:13" ht="261" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>55</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>122</v>
+      <c r="B2" t="s">
+        <v>75</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1244,42 +1103,42 @@
       <c r="F2" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>52</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>53</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="0">
+      <c r="M2">
         <v>20770</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51EBD9BD-D9A5-41D7-B0D1-A7DD8841A698}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51EBD9BD-D9A5-41D7-B0D1-A7DD8841A698}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="39.7265625" collapsed="true"/>
+    <col min="6" max="6" width="39.7265625" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1320,12 +1179,12 @@
         <v>18</v>
       </c>
     </row>
-    <row ht="159.5" r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:13" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>121</v>
+      <c r="B2" t="s">
+        <v>74</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1337,42 +1196,42 @@
       <c r="F2" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>52</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>53</v>
       </c>
       <c r="K2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="0">
+      <c r="M2">
         <v>20770</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DDB5A32-AE5F-4469-909E-B5CBB0B316F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DDB5A32-AE5F-4469-909E-B5CBB0B316F1}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="44.26953125" collapsed="true"/>
+    <col min="6" max="6" width="44.26953125" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1395,12 +1254,12 @@
         <v>50</v>
       </c>
     </row>
-    <row ht="116" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>125</v>
+      <c r="B2" t="s">
+        <v>73</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1412,26 +1271,26 @@
       <c r="F2" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDED305E-1D1F-4473-A9FE-10CCE4EF2A93}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDED305E-1D1F-4473-A9FE-10CCE4EF2A93}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="34.36328125" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" width="18.453125" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" width="22.0" collapsed="true"/>
+    <col min="6" max="6" width="34.36328125" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="18.453125" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="22" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="43.5" r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1466,12 +1325,12 @@
         <v>58</v>
       </c>
     </row>
-    <row ht="362.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:11" ht="362.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>126</v>
+      <c r="B2" t="s">
+        <v>83</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1485,7 +1344,7 @@
       </c>
       <c r="G2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>06/06/2026</v>
+        <v>08/26/2026</v>
       </c>
       <c r="H2" s="18">
         <v>10</v>
@@ -1502,29 +1361,29 @@
 Number of Payments:,Divide the Balance Due into ,
 Individual Amount:,Repeat this amount until the Balance Due is achieved: $, 
 Step 4: Review Payment Plan,
-1 Daily payment of $10.00 on 06/06/2026,A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 06/06/2026</v>
+1 Daily payment of $10.00 on 08/26/2026,A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 08/26/2026</v>
       </c>
       <c r="K2" s="14" t="str">
         <f ca="1">"A Convenience Fee will be added to each transaction issued for 1 Daily payment of "&amp;  TEXT(I2,"0.00")&amp;" starting on "&amp;G2</f>
-        <v>A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 06/06/2026</v>
+        <v>A Convenience Fee will be added to each transaction issued for 1 Daily payment of 0.00 starting on 08/26/2026</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4382B992-23F5-4C47-8E0D-617770DAB873}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4382B992-23F5-4C47-8E0D-617770DAB873}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="27.6328125" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" width="22.36328125" collapsed="true"/>
-    <col min="11" max="11" customWidth="true" width="25.7265625" collapsed="true"/>
+    <col min="6" max="6" width="27.6328125" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="22.36328125" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="25.7265625" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1559,12 +1418,12 @@
         <v>58</v>
       </c>
     </row>
-    <row ht="304.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:11" ht="304.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>130</v>
+      <c r="B2" t="s">
+        <v>79</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1578,7 +1437,7 @@
       </c>
       <c r="G2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>06/06/2026</v>
+        <v>08/26/2026</v>
       </c>
       <c r="H2" s="18">
         <v>10</v>
@@ -1592,7 +1451,7 @@
 Deferred,
 Select the date you wish to submit your payment,
 Step 4: Review Payment Plan,
-1 Deferred payment of $10.00 on 06/06/2026,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
+1 Deferred payment of $10.00 on 08/26/2026,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 08/26/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
@@ -1600,27 +1459,27 @@
         <f ca="1">"A Convenience Fee will be added to each transaction issued for 1 Deferred payment of "&amp;  TEXT(I2,"0.00")&amp;" starting on "&amp;G2&amp;" ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:"</f>
-        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
+        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 08/26/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EA3BF1-14B8-47AF-A2C8-3C7ED7468772}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EA3BF1-14B8-47AF-A2C8-3C7ED7468772}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="29.90625" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" width="29.453125" collapsed="true"/>
-    <col min="11" max="11" customWidth="true" width="22.7265625" collapsed="true"/>
+    <col min="6" max="6" width="29.90625" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="29.453125" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="22.7265625" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1655,12 +1514,12 @@
         <v>58</v>
       </c>
     </row>
-    <row ht="304.5" r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:11" ht="304.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>129</v>
+      <c r="B2" t="s">
+        <v>78</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1674,7 +1533,7 @@
       </c>
       <c r="G2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>06/06/2026</v>
+        <v>08/26/2026</v>
       </c>
       <c r="H2" s="18">
         <v>10</v>
@@ -1689,7 +1548,7 @@
 Daily,
 Select the date you wish to submit your first payment and it will recur every day after,
 Step 4: Review Payment Plan,
-Daily payments of $10.00 starting on 06/06/2026,A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
+Daily payments of $10.00 starting on 08/26/2026,A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 08/26/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
@@ -1697,22 +1556,22 @@
         <f ca="1">"A Convenience Fee will be added to each transaction issued for Daily payment of "&amp;  TEXT(I2,"0.00")&amp;" starting on "&amp;G2&amp;" ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:"</f>
-        <v>A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 06/06/2026 ,Individual Convenience Fee Amount:,	
+        <v>A Convenience Fee will be added to each transaction issued for Daily payment of 0.00 starting on 08/26/2026 ,Individual Convenience Fee Amount:,	
 Total Convenience Fees Paid:,	
 Total Paid under this plan:</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E59FD46A-A4BF-4EFF-8C85-302E7420C761}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E59FD46A-A4BF-4EFF-8C85-302E7420C761}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="40.54296875" collapsed="true"/>
+    <col min="6" max="6" width="40.54296875" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1735,12 +1594,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="101.5" r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>124</v>
+      <c r="B2" t="s">
+        <v>77</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1754,17 +1613,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D81D62B-D7FF-4418-A543-2CCEB8B27904}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D81D62B-D7FF-4418-A543-2CCEB8B27904}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="39.453125" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" width="40.1796875" collapsed="true"/>
+    <col min="6" max="6" width="39.453125" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="40.1796875" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1790,12 +1649,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="246.5" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:7" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>127</v>
+      <c r="B2" t="s">
+        <v>84</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1817,21 +1676,21 @@
 Number of Payments:,Divide the Balance Due into, 
 Individual Amount:,	Repeat this amount until the Balance Due is achieved: $ ,
 Step 4: Review Payment Plan
-1 Quarterly payment of $10.00 on 06/06/2026</v>
+1 Quarterly payment of $10.00 on 08/26/2026</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6951466-0A68-4F4C-8CFE-91C88774BAFD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6951466-0A68-4F4C-8CFE-91C88774BAFD}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="6" customWidth="true" width="53.6328125" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" width="41.0" collapsed="true"/>
+    <col min="6" max="6" width="53.6328125" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="41" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -1857,12 +1716,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="159.5" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>105</v>
+      <c r="B2" t="s">
+        <v>70</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -1881,21 +1740,21 @@
 Select the date you wish to submit your first payment and it will recur every year on that day,
 Divide your payment plan by...,
 Number of Payments:,Divide the Balance Due into,
-Individual Amount:,Repeat this amount until the Balance Due is achieved: $,1 Annual payment of $10.00 on 06/06/2026</v>
+Individual Amount:,Repeat this amount until the Balance Due is achieved: $,1 Annual payment of $10.00 on 08/26/2026</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F59C5AD-9583-4572-BF59-08E264185AA4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F59C5AD-9583-4572-BF59-08E264185AA4}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.81640625" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" width="11.08984375" collapsed="true"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="11.08984375" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -1934,38 +1793,38 @@
       <c r="C2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="0">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="F2" s="0">
+      <c r="F2">
         <v>1</v>
       </c>
-      <c r="G2" s="0">
+      <c r="G2">
         <v>3</v>
       </c>
-      <c r="H2" s="0">
+      <c r="H2">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{106EA5F4-3A74-4B88-9694-190DD754DB42}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{106EA5F4-3A74-4B88-9694-190DD754DB42}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" customWidth="true" width="35.54296875" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.453125" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="7.54296875" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" width="7.54296875" collapsed="true"/>
-    <col min="9" max="9" customWidth="true" width="29.54296875" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" width="31.26953125" collapsed="true"/>
+    <col min="5" max="5" width="35.54296875" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="7.54296875" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="7.54296875" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="29.54296875" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="31.26953125" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1997,12 +1856,12 @@
         <v>58</v>
       </c>
     </row>
-    <row ht="232" r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:10" ht="232" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>128</v>
+      <c r="B2" t="s">
+        <v>85</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2013,7 +1872,7 @@
       </c>
       <c r="F2" s="15" t="str">
         <f ca="1">TEXT(TODAY()+1,"mm/dd/yyyy")</f>
-        <v>06/06/2026</v>
+        <v>08/26/2026</v>
       </c>
       <c r="G2" s="18">
         <v>10</v>
@@ -2029,26 +1888,26 @@
  Individual Amount:,	Repeat this amount until the Balance Due is achieved: $, 
 10.00,
 Step 4: Review Payment Plan,
-1 Deferred payment of $10.00 on 06/06/2026,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026</v>
+1 Deferred payment of $10.00 on 08/26/2026,A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 08/26/2026</v>
       </c>
       <c r="J2" s="14" t="str">
         <f ca="1">"A Convenience Fee will be added to each transaction issued for 1 Deferred payment of "&amp;  TEXT(H2,"0.00")&amp;" starting on "&amp;F2</f>
-        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 06/06/2026</v>
+        <v>A Convenience Fee will be added to each transaction issued for 1 Deferred payment of 0.00 starting on 08/26/2026</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22FCBBA-7D6F-4A96-ABDF-B9688B9AD57A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C22FCBBA-7D6F-4A96-ABDF-B9688B9AD57A}">
   <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.7265625" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" width="16.1796875" collapsed="true"/>
-    <col min="11" max="11" customWidth="true" width="13.90625" collapsed="true"/>
+    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="16.1796875" customWidth="1" collapsed="1"/>
+    <col min="11" max="11" width="13.90625" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -2087,10 +1946,10 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="4"/>
@@ -2118,10 +1977,10 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>37</v>
       </c>
       <c r="C3" s="4"/>
@@ -2145,10 +2004,10 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="4"/>
@@ -2172,19 +2031,19 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2E036A-EB5C-429E-B5B6-2CEB663A49DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2E036A-EB5C-429E-B5B6-2CEB663A49DE}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="25.81640625" collapsed="true"/>
+    <col min="2" max="2" width="25.81640625" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row ht="29" r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2217,10 +2076,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>40</v>
       </c>
       <c r="C2" s="4"/>
@@ -2247,16 +2106,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8A1DA2-5F25-403C-A696-AD0A990EA2A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8A1DA2-5F25-403C-A696-AD0A990EA2A5}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row ht="29" r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2289,10 +2148,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>39</v>
       </c>
       <c r="C2" s="4"/>
@@ -2319,12 +2178,12 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3003305-5779-4E10-BB96-1E05DA55CF7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3003305-5779-4E10-BB96-1E05DA55CF7C}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -2357,12 +2216,12 @@
         <v>10</v>
       </c>
     </row>
-    <row ht="409.5" r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>123</v>
+      <c r="B2" t="s">
+        <v>76</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2385,16 +2244,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8EB073-2CB6-4360-AD8F-5A1F832738F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B8EB073-2CB6-4360-AD8F-5A1F832738F2}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="19.08984375" collapsed="true"/>
+    <col min="5" max="5" width="19.08984375" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -2415,11 +2274,11 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>100</v>
+      <c r="B2" t="s">
+        <v>69</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2430,12 +2289,12 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F658B4C-7DBB-4EDF-981E-97E4B7C1F375}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F658B4C-7DBB-4EDF-981E-97E4B7C1F375}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -2457,11 +2316,11 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>112</v>
+      <c r="B2" t="s">
+        <v>71</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2472,17 +2331,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C921207-0810-405F-8F16-4133FFE6EA23}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C921207-0810-405F-8F16-4133FFE6EA23}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="6" bestFit="true" customWidth="true" width="19.08984375" collapsed="true"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="68.1796875" collapsed="true"/>
+    <col min="5" max="6" width="19.08984375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="68.1796875" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -2508,12 +2367,12 @@
         <v>10</v>
       </c>
     </row>
-    <row customHeight="1" ht="52" r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+    <row r="2" spans="1:7" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>131</v>
+      <c r="B2" t="s">
+        <v>80</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
@@ -2522,48 +2381,48 @@
       <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="15" t="s">
         <v>49</v>
       </c>
     </row>
-    <row ht="29" r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" t="s" s="0">
-        <v>132</v>
-      </c>
-      <c r="D3" t="s" s="0">
+      <c r="B3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="15" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="D4" t="s" s="0">
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="E4" t="s">
         <v>48</v>
       </c>
-      <c r="G4" t="s" s="0">
+      <c r="G4" s="19" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>